<commit_message>
Actually using non-corrected Ex spectra for the angular distributions
</commit_message>
<xml_diff>
--- a/analysis/corrected_working/SF_17O17F_minuitfit.xlsx
+++ b/analysis/corrected_working/SF_17O17F_minuitfit.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10824"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kawecka/digios/analysis/corrected_working/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57671C07-089D-D948-BE8C-0C6EABFCB097}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC3DAFEE-31E9-AE4C-AD58-022876461066}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="17220" activeTab="2" xr2:uid="{CD653CE8-44FC-9042-84CB-1A005792DB96}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="17160" xr2:uid="{CD653CE8-44FC-9042-84CB-1A005792DB96}"/>
   </bookViews>
   <sheets>
     <sheet name="17O" sheetId="1" r:id="rId1"/>
     <sheet name="17F" sheetId="2" r:id="rId2"/>
     <sheet name="17F_scaled" sheetId="4" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="30">
   <si>
     <t>A</t>
   </si>
@@ -125,6 +125,9 @@
   </si>
   <si>
     <t>scaled to 17O (I compared the 1.982 MeV peak in oxygen with the 3.062 MeV peak in fluorine)</t>
+  </si>
+  <si>
+    <t>chi2</t>
   </si>
 </sst>
 </file>
@@ -336,7 +339,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
@@ -366,8 +369,6 @@
     <xf numFmtId="0" fontId="0" fillId="13" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -703,50 +704,48 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{418A8245-1A59-3C41-BCB4-A6C2419E4CFE}">
-  <dimension ref="B1:Y39"/>
+  <dimension ref="B1:AB39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3.1640625" customWidth="1"/>
     <col min="2" max="2" width="3.5" customWidth="1"/>
     <col min="3" max="3" width="3.33203125" customWidth="1"/>
-    <col min="20" max="20" width="12.1640625" customWidth="1"/>
+    <col min="22" max="22" width="12.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:25" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:25" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:28" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="D2" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="29"/>
-      <c r="M2" s="28" t="s">
+      <c r="N2" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="N2" s="29"/>
-      <c r="V2" s="28" t="s">
+      <c r="X2" s="28" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:28" x14ac:dyDescent="0.2">
       <c r="D3" t="s">
         <v>15</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>16</v>
       </c>
-      <c r="M3" t="s">
+      <c r="N3" t="s">
         <v>15</v>
       </c>
-      <c r="R3" t="s">
+      <c r="T3" t="s">
         <v>16</v>
       </c>
-      <c r="V3" t="s">
+      <c r="X3" t="s">
         <v>15</v>
       </c>
-      <c r="X3" t="s">
+      <c r="AA3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:28" x14ac:dyDescent="0.2">
       <c r="D4" s="27" t="s">
         <v>12</v>
       </c>
@@ -760,55 +759,64 @@
         <v>22</v>
       </c>
       <c r="H4" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="I4" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="27" t="s">
+      <c r="J4" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="J4" s="27" t="s">
+      <c r="K4" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="K4" s="27" t="s">
+      <c r="L4" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="M4" s="27" t="s">
+      <c r="N4" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="N4" s="27" t="s">
+      <c r="O4" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="O4" s="27" t="s">
+      <c r="P4" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="P4" s="27" t="s">
+      <c r="Q4" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="Q4" s="27" t="s">
+      <c r="R4" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="S4" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="R4" s="27" t="s">
+      <c r="T4" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="S4" s="27" t="s">
+      <c r="U4" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="T4" s="27" t="s">
+      <c r="V4" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="V4" s="27" t="s">
+      <c r="X4" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="W4" s="30" t="s">
+      <c r="Y4" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="X4" s="30" t="s">
+      <c r="Z4" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="AA4" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="Y4" s="30" t="s">
+      <c r="AB4" s="27" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:28" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
         <v>0</v>
       </c>
@@ -827,44 +835,57 @@
       <c r="G5">
         <v>0.81089900000000004</v>
       </c>
-      <c r="I5" s="31">
+      <c r="H5">
+        <v>0.74683699999999997</v>
+      </c>
+      <c r="I5">
+        <f>D5/F5</f>
+        <v>0.13320688210794193</v>
+      </c>
+      <c r="J5" s="29">
         <v>0.21</v>
       </c>
-      <c r="J5">
+      <c r="K5">
         <v>0.83</v>
       </c>
-      <c r="M5">
+      <c r="N5">
         <v>1.4817499999999999</v>
       </c>
-      <c r="N5">
+      <c r="O5">
         <v>0.54227300000000001</v>
       </c>
-      <c r="O5">
+      <c r="P5">
         <v>3.4672200000000002</v>
       </c>
-      <c r="P5">
+      <c r="Q5">
         <v>0.73882700000000001</v>
       </c>
-      <c r="R5" s="31">
+      <c r="R5">
+        <v>3.3786700000000001</v>
+      </c>
+      <c r="T5" s="29">
         <v>0.35</v>
       </c>
-      <c r="S5">
+      <c r="U5">
         <v>0.66</v>
       </c>
-      <c r="V5">
+      <c r="X5">
         <v>8.1363699999999994</v>
       </c>
-      <c r="W5">
+      <c r="Y5">
         <v>0.50545499999999999</v>
       </c>
-      <c r="X5" s="31">
+      <c r="Z5">
+        <v>4.9880599999999999</v>
+      </c>
+      <c r="AA5" s="29">
         <v>1.57</v>
       </c>
-      <c r="Y5">
+      <c r="AB5">
         <v>0.28000000000000003</v>
       </c>
     </row>
-    <row r="6" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:28" x14ac:dyDescent="0.2">
       <c r="B6" s="3" t="s">
         <v>0</v>
       </c>
@@ -883,26 +904,35 @@
       <c r="G6">
         <v>0.85338700000000001</v>
       </c>
-      <c r="M6">
+      <c r="H6">
+        <v>0.74424699999999999</v>
+      </c>
+      <c r="N6">
         <v>1.4068099999999999</v>
       </c>
-      <c r="N6">
+      <c r="O6">
         <v>0.56330899999999995</v>
       </c>
-      <c r="O6">
+      <c r="P6">
         <v>3.7296999999999998</v>
       </c>
-      <c r="P6">
+      <c r="Q6">
         <v>0.77150099999999999</v>
       </c>
-      <c r="V6">
+      <c r="R6">
+        <v>3.9870800000000002</v>
+      </c>
+      <c r="X6">
         <v>8.4337300000000006</v>
       </c>
-      <c r="W6">
+      <c r="Y6">
         <v>0.52318399999999998</v>
       </c>
-    </row>
-    <row r="7" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="Z6">
+        <v>4.2529500000000002</v>
+      </c>
+    </row>
+    <row r="7" spans="2:28" x14ac:dyDescent="0.2">
       <c r="B7" s="3" t="s">
         <v>0</v>
       </c>
@@ -921,26 +951,35 @@
       <c r="G7">
         <v>0.91736700000000004</v>
       </c>
-      <c r="M7">
+      <c r="H7">
+        <v>0.79306200000000004</v>
+      </c>
+      <c r="N7">
         <v>1.49773</v>
       </c>
-      <c r="N7">
+      <c r="O7">
         <v>0.53899799999999998</v>
       </c>
-      <c r="O7">
+      <c r="P7">
         <v>4.0827900000000001</v>
       </c>
-      <c r="P7">
+      <c r="Q7">
         <v>0.81062500000000004</v>
       </c>
-      <c r="V7">
+      <c r="R7">
+        <v>3.47804</v>
+      </c>
+      <c r="X7">
         <v>9.3617899999999992</v>
       </c>
-      <c r="W7">
+      <c r="Y7">
         <v>0.58193899999999998</v>
       </c>
-    </row>
-    <row r="8" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="Z7">
+        <v>5.3164300000000004</v>
+      </c>
+    </row>
+    <row r="8" spans="2:28" x14ac:dyDescent="0.2">
       <c r="B8" s="3" t="s">
         <v>0</v>
       </c>
@@ -959,26 +998,35 @@
       <c r="G8">
         <v>0.89912599999999998</v>
       </c>
-      <c r="M8">
+      <c r="H8">
+        <v>0.76234000000000002</v>
+      </c>
+      <c r="N8">
         <v>1.54251</v>
       </c>
-      <c r="N8">
+      <c r="O8">
         <v>0.54468499999999997</v>
       </c>
-      <c r="O8">
+      <c r="P8">
         <v>3.8130500000000001</v>
       </c>
-      <c r="P8">
+      <c r="Q8">
         <v>0.79746700000000004</v>
       </c>
-      <c r="V8">
+      <c r="R8">
+        <v>3.3515999999999999</v>
+      </c>
+      <c r="X8">
         <v>9.0026399999999995</v>
       </c>
-      <c r="W8">
+      <c r="Y8">
         <v>0.55986400000000003</v>
       </c>
-    </row>
-    <row r="9" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="Z8">
+        <v>5.5448300000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="2:28" x14ac:dyDescent="0.2">
       <c r="B9" s="7" t="s">
         <v>0</v>
       </c>
@@ -997,26 +1045,35 @@
       <c r="G9">
         <v>0.85477300000000001</v>
       </c>
-      <c r="M9">
+      <c r="H9">
+        <v>0.67946700000000004</v>
+      </c>
+      <c r="N9">
         <v>1.6323099999999999</v>
       </c>
-      <c r="N9">
+      <c r="O9">
         <v>0.56235400000000002</v>
       </c>
-      <c r="O9">
+      <c r="P9">
         <v>3.39201</v>
       </c>
-      <c r="P9">
+      <c r="Q9">
         <v>0.77291100000000001</v>
       </c>
-      <c r="V9">
+      <c r="R9">
+        <v>2.9304899999999998</v>
+      </c>
+      <c r="X9">
         <v>8.3710000000000004</v>
       </c>
-      <c r="W9">
+      <c r="Y9">
         <v>0.52062600000000003</v>
       </c>
-    </row>
-    <row r="10" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="Z9">
+        <v>5.5821199999999997</v>
+      </c>
+    </row>
+    <row r="10" spans="2:28" x14ac:dyDescent="0.2">
       <c r="B10" s="9" t="s">
         <v>6</v>
       </c>
@@ -1035,26 +1092,35 @@
       <c r="G10">
         <v>0.71857599999999999</v>
       </c>
-      <c r="M10">
+      <c r="H10">
+        <v>0.71196999999999999</v>
+      </c>
+      <c r="N10">
         <v>1.35893</v>
       </c>
-      <c r="N10">
+      <c r="O10">
         <v>0.463065</v>
       </c>
-      <c r="O10">
+      <c r="P10">
         <v>3.2860800000000001</v>
       </c>
-      <c r="P10">
+      <c r="Q10">
         <v>0.63619800000000004</v>
       </c>
-      <c r="V10">
+      <c r="R10">
+        <v>2.2158600000000002</v>
+      </c>
+      <c r="X10">
         <v>7.5032899999999998</v>
       </c>
-      <c r="W10">
+      <c r="Y10">
         <v>0.46621699999999999</v>
       </c>
-    </row>
-    <row r="11" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="Z10">
+        <v>5.0050299999999996</v>
+      </c>
+    </row>
+    <row r="11" spans="2:28" x14ac:dyDescent="0.2">
       <c r="B11" s="10" t="s">
         <v>6</v>
       </c>
@@ -1073,26 +1139,35 @@
       <c r="G11">
         <v>0.75768999999999997</v>
       </c>
-      <c r="M11">
+      <c r="H11">
+        <v>0.69737199999999999</v>
+      </c>
+      <c r="N11">
         <v>1.34206</v>
       </c>
-      <c r="N11">
+      <c r="O11">
         <v>0.48949100000000001</v>
       </c>
-      <c r="O11">
+      <c r="P11">
         <v>3.47472</v>
       </c>
-      <c r="P11">
+      <c r="Q11">
         <v>0.67097899999999999</v>
       </c>
-      <c r="V11">
+      <c r="R11">
+        <v>2.6364000000000001</v>
+      </c>
+      <c r="X11">
         <v>7.7808999999999999</v>
       </c>
-      <c r="W11">
+      <c r="Y11">
         <v>0.48270299999999999</v>
       </c>
-    </row>
-    <row r="12" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="Z11">
+        <v>4.2670199999999996</v>
+      </c>
+    </row>
+    <row r="12" spans="2:28" x14ac:dyDescent="0.2">
       <c r="B12" s="10" t="s">
         <v>6</v>
       </c>
@@ -1111,26 +1186,35 @@
       <c r="G12">
         <v>0.81475500000000001</v>
       </c>
-      <c r="M12">
+      <c r="H12">
+        <v>0.77593500000000004</v>
+      </c>
+      <c r="N12">
         <v>1.3650599999999999</v>
       </c>
-      <c r="N12">
+      <c r="O12">
         <v>0.46379500000000001</v>
       </c>
-      <c r="O12">
+      <c r="P12">
         <v>3.8128700000000002</v>
       </c>
-      <c r="P12">
+      <c r="Q12">
         <v>0.70629399999999998</v>
       </c>
-      <c r="V12">
+      <c r="R12">
+        <v>2.2953000000000001</v>
+      </c>
+      <c r="X12">
         <v>8.55898</v>
       </c>
-      <c r="W12">
+      <c r="Y12">
         <v>0.531914</v>
       </c>
-    </row>
-    <row r="13" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="Z12">
+        <v>5.1918300000000004</v>
+      </c>
+    </row>
+    <row r="13" spans="2:28" x14ac:dyDescent="0.2">
       <c r="B13" s="10" t="s">
         <v>6</v>
       </c>
@@ -1149,26 +1233,35 @@
       <c r="G13">
         <v>0.79260799999999998</v>
       </c>
-      <c r="M13">
+      <c r="H13">
+        <v>0.73689499999999997</v>
+      </c>
+      <c r="N13">
         <v>1.4028499999999999</v>
       </c>
-      <c r="N13">
+      <c r="O13">
         <v>0.46204499999999998</v>
       </c>
-      <c r="O13">
+      <c r="P13">
         <v>3.59396</v>
       </c>
-      <c r="P13">
+      <c r="Q13">
         <v>0.685809</v>
       </c>
-      <c r="V13">
+      <c r="R13">
+        <v>2.2172700000000001</v>
+      </c>
+      <c r="X13">
         <v>8.2650600000000001</v>
       </c>
-      <c r="W13">
+      <c r="Y13">
         <v>0.51411899999999999</v>
       </c>
-    </row>
-    <row r="14" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="Z13">
+        <v>5.6628499999999997</v>
+      </c>
+    </row>
+    <row r="14" spans="2:28" x14ac:dyDescent="0.2">
       <c r="B14" s="11" t="s">
         <v>6</v>
       </c>
@@ -1187,26 +1280,35 @@
       <c r="G14">
         <v>0.74349100000000001</v>
       </c>
-      <c r="M14">
+      <c r="H14">
+        <v>0.65632599999999996</v>
+      </c>
+      <c r="N14">
         <v>1.4626999999999999</v>
       </c>
-      <c r="N14">
+      <c r="O14">
         <v>0.471798</v>
       </c>
-      <c r="O14">
+      <c r="P14">
         <v>3.2350300000000001</v>
       </c>
-      <c r="P14">
+      <c r="Q14">
         <v>0.653613</v>
       </c>
-      <c r="V14">
+      <c r="R14">
+        <v>1.9373499999999999</v>
+      </c>
+      <c r="X14">
         <v>7.6701600000000001</v>
       </c>
-      <c r="W14">
+      <c r="Y14">
         <v>0.47722399999999998</v>
       </c>
-    </row>
-    <row r="15" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="Z14">
+        <v>5.7819000000000003</v>
+      </c>
+    </row>
+    <row r="15" spans="2:28" x14ac:dyDescent="0.2">
       <c r="B15" s="12" t="s">
         <v>7</v>
       </c>
@@ -1225,26 +1327,35 @@
       <c r="G15">
         <v>0.77404300000000004</v>
       </c>
-      <c r="M15">
+      <c r="H15">
+        <v>0.78478599999999998</v>
+      </c>
+      <c r="N15">
         <v>1.4231199999999999</v>
       </c>
-      <c r="N15">
+      <c r="O15">
         <v>0.45355000000000001</v>
       </c>
-      <c r="O15">
+      <c r="P15">
         <v>3.4855200000000002</v>
       </c>
-      <c r="P15">
+      <c r="Q15">
         <v>0.68437099999999995</v>
       </c>
-      <c r="V15">
+      <c r="R15">
+        <v>1.92117</v>
+      </c>
+      <c r="X15">
         <v>8.18675</v>
       </c>
-      <c r="W15">
+      <c r="Y15">
         <v>0.50970700000000002</v>
       </c>
-    </row>
-    <row r="16" spans="2:25" x14ac:dyDescent="0.2">
+      <c r="Z15">
+        <v>6.1279399999999997</v>
+      </c>
+    </row>
+    <row r="16" spans="2:28" x14ac:dyDescent="0.2">
       <c r="B16" s="13" t="s">
         <v>7</v>
       </c>
@@ -1263,26 +1374,35 @@
       <c r="G16">
         <v>0.81630999999999998</v>
       </c>
-      <c r="M16">
+      <c r="H16">
+        <v>0.75895999999999997</v>
+      </c>
+      <c r="N16">
         <v>1.4352400000000001</v>
       </c>
-      <c r="N16">
+      <c r="O16">
         <v>0.48338799999999998</v>
       </c>
-      <c r="O16">
+      <c r="P16">
         <v>3.6794600000000002</v>
       </c>
-      <c r="P16">
+      <c r="Q16">
         <v>0.72297900000000004</v>
       </c>
-      <c r="V16">
+      <c r="R16">
+        <v>2.3372899999999999</v>
+      </c>
+      <c r="X16">
         <v>8.5122900000000001</v>
       </c>
-      <c r="W16">
+      <c r="Y16">
         <v>0.52914399999999995</v>
       </c>
-    </row>
-    <row r="17" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="Z16">
+        <v>5.3200700000000003</v>
+      </c>
+    </row>
+    <row r="17" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B17" s="13" t="s">
         <v>7</v>
       </c>
@@ -1301,26 +1421,35 @@
       <c r="G17">
         <v>0.88157600000000003</v>
       </c>
-      <c r="M17">
+      <c r="H17">
+        <v>0.88670499999999997</v>
+      </c>
+      <c r="N17">
         <v>1.4409400000000001</v>
       </c>
-      <c r="N17">
+      <c r="O17">
         <v>0.45332600000000001</v>
       </c>
-      <c r="O17">
+      <c r="P17">
         <v>4.0978300000000001</v>
       </c>
-      <c r="P17">
+      <c r="Q17">
         <v>0.75816399999999995</v>
       </c>
-      <c r="V17">
+      <c r="R17">
+        <v>2.0165899999999999</v>
+      </c>
+      <c r="X17">
         <v>9.4137500000000003</v>
       </c>
-      <c r="W17">
+      <c r="Y17">
         <v>0.58655299999999999</v>
       </c>
-    </row>
-    <row r="18" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="Z17">
+        <v>6.5362600000000004</v>
+      </c>
+    </row>
+    <row r="18" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B18" s="13" t="s">
         <v>7</v>
       </c>
@@ -1339,26 +1468,35 @@
       <c r="G18">
         <v>0.85948999999999998</v>
       </c>
-      <c r="M18">
+      <c r="H18">
+        <v>0.83178600000000003</v>
+      </c>
+      <c r="N18">
         <v>1.4698100000000001</v>
       </c>
-      <c r="N18">
+      <c r="O18">
         <v>0.45387699999999997</v>
       </c>
-      <c r="O18">
+      <c r="P18">
         <v>3.8424299999999998</v>
       </c>
-      <c r="P18">
+      <c r="Q18">
         <v>0.74008099999999999</v>
       </c>
-      <c r="V18">
+      <c r="R18">
+        <v>1.9354199999999999</v>
+      </c>
+      <c r="X18">
         <v>9.0603700000000007</v>
       </c>
-      <c r="W18">
+      <c r="Y18">
         <v>0.56495099999999998</v>
       </c>
-    </row>
-    <row r="19" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="Z18">
+        <v>6.9137300000000002</v>
+      </c>
+    </row>
+    <row r="19" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B19" s="14" t="s">
         <v>7</v>
       </c>
@@ -1377,26 +1515,35 @@
       <c r="G19">
         <v>0.81272</v>
       </c>
-      <c r="M19">
+      <c r="H19">
+        <v>0.71602299999999997</v>
+      </c>
+      <c r="N19">
         <v>1.5207900000000001</v>
       </c>
-      <c r="N19">
+      <c r="O19">
         <v>0.46424300000000002</v>
       </c>
-      <c r="O19">
+      <c r="P19">
         <v>3.4607000000000001</v>
       </c>
-      <c r="P19">
+      <c r="Q19">
         <v>0.71184499999999995</v>
       </c>
-      <c r="V19">
+      <c r="R19">
+        <v>1.6994</v>
+      </c>
+      <c r="X19">
         <v>8.4406199999999991</v>
       </c>
-      <c r="W19">
+      <c r="Y19">
         <v>0.52633099999999999</v>
       </c>
-    </row>
-    <row r="20" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="Z19">
+        <v>6.9316500000000003</v>
+      </c>
+    </row>
+    <row r="20" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B20" s="15" t="s">
         <v>8</v>
       </c>
@@ -1415,26 +1562,35 @@
       <c r="G20">
         <v>0.75117900000000004</v>
       </c>
-      <c r="M20">
+      <c r="H20">
+        <v>0.71354700000000004</v>
+      </c>
+      <c r="N20">
         <v>1.3349800000000001</v>
       </c>
-      <c r="N20">
+      <c r="O20">
         <v>0.49672300000000003</v>
       </c>
-      <c r="O20">
+      <c r="P20">
         <v>3.33582</v>
       </c>
-      <c r="P20">
+      <c r="Q20">
         <v>0.68774500000000005</v>
       </c>
-      <c r="V20">
+      <c r="R20">
+        <v>2.7793100000000002</v>
+      </c>
+      <c r="X20">
         <v>7.6313500000000003</v>
       </c>
-      <c r="W20">
+      <c r="Y20">
         <v>0.47350300000000001</v>
       </c>
-    </row>
-    <row r="21" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="Z20">
+        <v>4.3535399999999997</v>
+      </c>
+    </row>
+    <row r="21" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B21" s="16" t="s">
         <v>8</v>
       </c>
@@ -1453,26 +1609,35 @@
       <c r="G21">
         <v>0.79089399999999999</v>
       </c>
-      <c r="M21">
+      <c r="H21">
+        <v>0.698291</v>
+      </c>
+      <c r="N21">
         <v>1.28081</v>
       </c>
-      <c r="N21">
+      <c r="O21">
         <v>0.51881299999999997</v>
       </c>
-      <c r="O21">
+      <c r="P21">
         <v>3.5668500000000001</v>
       </c>
-      <c r="P21">
+      <c r="Q21">
         <v>0.71994100000000005</v>
       </c>
-      <c r="V21">
+      <c r="R21">
+        <v>3.2720400000000001</v>
+      </c>
+      <c r="X21">
         <v>7.90381</v>
       </c>
-      <c r="W21">
+      <c r="Y21">
         <v>0.48980099999999999</v>
       </c>
-    </row>
-    <row r="22" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="Z21">
+        <v>3.7082799999999998</v>
+      </c>
+    </row>
+    <row r="22" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B22" s="16" t="s">
         <v>8</v>
       </c>
@@ -1491,26 +1656,35 @@
       <c r="G22">
         <v>0.845997</v>
       </c>
-      <c r="M22">
+      <c r="H22">
+        <v>0.76057900000000001</v>
+      </c>
+      <c r="N22">
         <v>1.3472</v>
       </c>
-      <c r="N22">
+      <c r="O22">
         <v>0.49517800000000001</v>
       </c>
-      <c r="O22">
+      <c r="P22">
         <v>3.9073199999999999</v>
       </c>
-      <c r="P22">
+      <c r="Q22">
         <v>0.75369399999999998</v>
       </c>
-      <c r="V22">
+      <c r="R22">
+        <v>2.8984299999999998</v>
+      </c>
+      <c r="X22">
         <v>8.7415599999999998</v>
       </c>
-      <c r="W22">
+      <c r="Y22">
         <v>0.54263899999999998</v>
       </c>
-    </row>
-    <row r="23" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="Z22">
+        <v>4.5995900000000001</v>
+      </c>
+    </row>
+    <row r="23" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B23" s="16" t="s">
         <v>8</v>
       </c>
@@ -1529,26 +1703,35 @@
       <c r="G23">
         <v>0.82906000000000002</v>
       </c>
-      <c r="M23">
+      <c r="H23">
+        <v>0.73532399999999998</v>
+      </c>
+      <c r="N23">
         <v>1.3828199999999999</v>
       </c>
-      <c r="N23">
+      <c r="O23">
         <v>0.49902200000000002</v>
       </c>
-      <c r="O23">
+      <c r="P23">
         <v>3.6680100000000002</v>
       </c>
-      <c r="P23">
+      <c r="Q23">
         <v>0.74088699999999996</v>
       </c>
-      <c r="V23">
+      <c r="R23">
+        <v>2.7820499999999999</v>
+      </c>
+      <c r="X23">
         <v>8.4204899999999991</v>
       </c>
-      <c r="W23">
+      <c r="Y23">
         <v>0.522926</v>
       </c>
-    </row>
-    <row r="24" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="Z23">
+        <v>4.81264</v>
+      </c>
+    </row>
+    <row r="24" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B24" s="17" t="s">
         <v>8</v>
       </c>
@@ -1556,7 +1739,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="2:23" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B25" s="18" t="s">
         <v>9</v>
       </c>
@@ -1564,7 +1747,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="2:23" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B26" s="19" t="s">
         <v>9</v>
       </c>
@@ -1572,7 +1755,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="2:23" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B27" s="19" t="s">
         <v>9</v>
       </c>
@@ -1591,26 +1774,35 @@
       <c r="G27">
         <v>1.37815</v>
       </c>
-      <c r="M27">
+      <c r="H27">
+        <v>0.74798699999999996</v>
+      </c>
+      <c r="N27">
         <v>1.36063</v>
       </c>
-      <c r="N27">
+      <c r="O27">
         <v>0.65990599999999999</v>
       </c>
-      <c r="O27">
+      <c r="P27">
         <v>5.9715600000000002</v>
       </c>
-      <c r="P27">
+      <c r="Q27">
         <v>1.08029</v>
       </c>
-      <c r="V27">
+      <c r="R27">
+        <v>4.5394399999999999</v>
+      </c>
+      <c r="X27">
         <v>12.2644</v>
       </c>
-      <c r="W27">
+      <c r="Y27">
         <v>0.75732600000000005</v>
       </c>
-    </row>
-    <row r="28" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="Z27">
+        <v>1.8796999999999999</v>
+      </c>
+    </row>
+    <row r="28" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B28" s="19" t="s">
         <v>9</v>
       </c>
@@ -1618,7 +1810,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="29" spans="2:23" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B29" s="20" t="s">
         <v>9</v>
       </c>
@@ -1626,7 +1818,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="2:23" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B30" s="21" t="s">
         <v>10</v>
       </c>
@@ -1645,26 +1837,35 @@
       <c r="G30">
         <v>0.96541200000000005</v>
       </c>
-      <c r="M30">
+      <c r="H30">
+        <v>0.69325400000000004</v>
+      </c>
+      <c r="N30">
         <v>1.63771</v>
       </c>
-      <c r="N30">
+      <c r="O30">
         <v>0.56880299999999995</v>
       </c>
-      <c r="O30">
+      <c r="P30">
         <v>4.0587499999999999</v>
       </c>
-      <c r="P30">
+      <c r="Q30">
         <v>0.82269000000000003</v>
       </c>
-      <c r="V30">
+      <c r="R30">
+        <v>2.9468700000000001</v>
+      </c>
+      <c r="X30">
         <v>9.4829899999999991</v>
       </c>
-      <c r="W30">
+      <c r="Y30">
         <v>0.58910499999999999</v>
       </c>
-    </row>
-    <row r="31" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="Z30">
+        <v>4.9925499999999996</v>
+      </c>
+    </row>
+    <row r="31" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B31" s="22" t="s">
         <v>10</v>
       </c>
@@ -1683,26 +1884,35 @@
       <c r="G31">
         <v>1.0113000000000001</v>
       </c>
-      <c r="M31">
+      <c r="H31">
+        <v>0.690079</v>
+      </c>
+      <c r="N31">
         <v>1.5822499999999999</v>
       </c>
-      <c r="N31">
+      <c r="O31">
         <v>0.59236900000000003</v>
       </c>
-      <c r="O31">
+      <c r="P31">
         <v>4.3089000000000004</v>
       </c>
-      <c r="P31">
+      <c r="Q31">
         <v>0.85857399999999995</v>
       </c>
-      <c r="V31">
+      <c r="R31">
+        <v>3.4666899999999998</v>
+      </c>
+      <c r="X31">
         <v>9.7856299999999994</v>
       </c>
-      <c r="W31">
+      <c r="Y31">
         <v>0.60696300000000003</v>
       </c>
-    </row>
-    <row r="32" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="Z31">
+        <v>4.1883499999999998</v>
+      </c>
+    </row>
+    <row r="32" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B32" s="22" t="s">
         <v>10</v>
       </c>
@@ -1721,26 +1931,35 @@
       <c r="G32">
         <v>1.0860300000000001</v>
       </c>
-      <c r="M32">
+      <c r="H32">
+        <v>0.72300200000000003</v>
+      </c>
+      <c r="N32">
         <v>1.6309800000000001</v>
       </c>
-      <c r="N32">
+      <c r="O32">
         <v>0.56778700000000004</v>
       </c>
-      <c r="O32">
+      <c r="P32">
         <v>4.7010500000000004</v>
       </c>
-      <c r="P32">
+      <c r="Q32">
         <v>0.90267600000000003</v>
       </c>
-      <c r="V32">
+      <c r="R32">
+        <v>2.9799500000000001</v>
+      </c>
+      <c r="X32">
         <v>10.725199999999999</v>
       </c>
-      <c r="W32">
+      <c r="Y32">
         <v>0.66628500000000002</v>
       </c>
-    </row>
-    <row r="33" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="Z32">
+        <v>4.9996099999999997</v>
+      </c>
+    </row>
+    <row r="33" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B33" s="22" t="s">
         <v>10</v>
       </c>
@@ -1759,26 +1978,35 @@
       <c r="G33">
         <v>1.0619000000000001</v>
       </c>
-      <c r="M33">
+      <c r="H33">
+        <v>0.69803999999999999</v>
+      </c>
+      <c r="N33">
         <v>1.7027300000000001</v>
       </c>
-      <c r="N33">
+      <c r="O33">
         <v>0.56806900000000005</v>
       </c>
-      <c r="O33">
+      <c r="P33">
         <v>4.4110500000000004</v>
       </c>
-      <c r="P33">
+      <c r="Q33">
         <v>0.88282000000000005</v>
       </c>
-      <c r="V33">
+      <c r="R33">
+        <v>2.96068</v>
+      </c>
+      <c r="X33">
         <v>10.4117</v>
       </c>
-      <c r="W33">
+      <c r="Y33">
         <v>0.64776800000000001</v>
       </c>
-    </row>
-    <row r="34" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="Z33">
+        <v>5.7698200000000002</v>
+      </c>
+    </row>
+    <row r="34" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B34" s="23" t="s">
         <v>10</v>
       </c>
@@ -1797,26 +2025,35 @@
       <c r="G34">
         <v>1.0007200000000001</v>
       </c>
-      <c r="M34">
+      <c r="H34">
+        <v>0.64625500000000002</v>
+      </c>
+      <c r="N34">
         <v>1.7754700000000001</v>
       </c>
-      <c r="N34">
+      <c r="O34">
         <v>0.58103199999999999</v>
       </c>
-      <c r="O34">
+      <c r="P34">
         <v>3.9734600000000002</v>
       </c>
-      <c r="P34">
+      <c r="Q34">
         <v>0.84673699999999996</v>
       </c>
-      <c r="V34">
+      <c r="R34">
+        <v>2.5621100000000001</v>
+      </c>
+      <c r="X34">
         <v>9.6873100000000001</v>
       </c>
-      <c r="W34">
+      <c r="Y34">
         <v>0.602746</v>
       </c>
-    </row>
-    <row r="35" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="Z34">
+        <v>5.8084199999999999</v>
+      </c>
+    </row>
+    <row r="35" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B35" s="24" t="s">
         <v>11</v>
       </c>
@@ -1835,26 +2072,35 @@
       <c r="G35">
         <v>0.78518200000000005</v>
       </c>
-      <c r="M35">
+      <c r="H35">
+        <v>1.13489</v>
+      </c>
+      <c r="N35">
         <v>1.57473</v>
       </c>
-      <c r="N35">
+      <c r="O35">
         <v>0.45174500000000001</v>
       </c>
-      <c r="O35">
+      <c r="P35">
         <v>3.4841199999999999</v>
       </c>
-      <c r="P35">
+      <c r="Q35">
         <v>0.68129899999999999</v>
       </c>
-      <c r="V35">
+      <c r="R35">
+        <v>1.9382299999999999</v>
+      </c>
+      <c r="X35">
         <v>8.4788700000000006</v>
       </c>
-      <c r="W35">
+      <c r="Y35">
         <v>0.53142</v>
       </c>
-    </row>
-    <row r="36" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="Z35">
+        <v>9.5424900000000008</v>
+      </c>
+    </row>
+    <row r="36" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B36" s="25" t="s">
         <v>11</v>
       </c>
@@ -1873,26 +2119,35 @@
       <c r="G36">
         <v>0.83075500000000002</v>
       </c>
-      <c r="M36">
+      <c r="H36">
+        <v>1.0952999999999999</v>
+      </c>
+      <c r="N36">
         <v>1.62418</v>
       </c>
-      <c r="N36">
+      <c r="O36">
         <v>0.486539</v>
       </c>
-      <c r="O36">
+      <c r="P36">
         <v>3.66934</v>
       </c>
-      <c r="P36">
+      <c r="Q36">
         <v>0.72451100000000002</v>
       </c>
-      <c r="V36">
+      <c r="R36">
+        <v>2.4533800000000001</v>
+      </c>
+      <c r="X36">
         <v>8.8715100000000007</v>
       </c>
-      <c r="W36">
+      <c r="Y36">
         <v>0.55510000000000004</v>
       </c>
-    </row>
-    <row r="37" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="Z36">
+        <v>8.69299</v>
+      </c>
+    </row>
+    <row r="37" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B37" s="25" t="s">
         <v>11</v>
       </c>
@@ -1911,26 +2166,35 @@
       <c r="G37">
         <v>0.90236099999999997</v>
       </c>
-      <c r="M37">
+      <c r="H37">
+        <v>1.43987</v>
+      </c>
+      <c r="N37">
         <v>1.5945199999999999</v>
       </c>
-      <c r="N37">
+      <c r="O37">
         <v>0.452239</v>
       </c>
-      <c r="O37">
+      <c r="P37">
         <v>4.1391999999999998</v>
       </c>
-      <c r="P37">
+      <c r="Q37">
         <v>0.76180800000000004</v>
       </c>
-      <c r="V37">
+      <c r="R37">
+        <v>2.06447</v>
+      </c>
+      <c r="X37">
         <v>9.8178599999999996</v>
       </c>
-      <c r="W37">
+      <c r="Y37">
         <v>0.61617599999999995</v>
       </c>
-    </row>
-    <row r="38" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="Z37">
+        <v>10.238200000000001</v>
+      </c>
+    </row>
+    <row r="38" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B38" s="25" t="s">
         <v>11</v>
       </c>
@@ -1949,26 +2213,35 @@
       <c r="G38">
         <v>0.869089</v>
       </c>
-      <c r="M38">
+      <c r="H38">
+        <v>1.2638499999999999</v>
+      </c>
+      <c r="N38">
         <v>1.61802</v>
       </c>
-      <c r="N38">
+      <c r="O38">
         <v>0.45091599999999998</v>
       </c>
-      <c r="O38">
+      <c r="P38">
         <v>3.8262</v>
       </c>
-      <c r="P38">
+      <c r="Q38">
         <v>0.73281200000000002</v>
       </c>
-      <c r="V38">
+      <c r="R38">
+        <v>1.92954</v>
+      </c>
+      <c r="X38">
         <v>9.3289299999999997</v>
       </c>
-      <c r="W38">
+      <c r="Y38">
         <v>0.58593600000000001</v>
       </c>
-    </row>
-    <row r="39" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="Z38">
+        <v>10.6236</v>
+      </c>
+    </row>
+    <row r="39" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B39" s="26" t="s">
         <v>11</v>
       </c>
@@ -1987,23 +2260,32 @@
       <c r="G39">
         <v>0.81704200000000005</v>
       </c>
-      <c r="M39">
+      <c r="H39">
+        <v>0.97375699999999998</v>
+      </c>
+      <c r="N39">
         <v>1.6464099999999999</v>
       </c>
-      <c r="N39">
+      <c r="O39">
         <v>0.46002799999999999</v>
       </c>
-      <c r="O39">
+      <c r="P39">
         <v>3.4353199999999999</v>
       </c>
-      <c r="P39">
+      <c r="Q39">
         <v>0.69856799999999997</v>
       </c>
-      <c r="V39">
+      <c r="R39">
+        <v>1.6388799999999999</v>
+      </c>
+      <c r="X39">
         <v>8.6178699999999999</v>
       </c>
-      <c r="W39">
+      <c r="Y39">
         <v>0.54074999999999995</v>
+      </c>
+      <c r="Z39">
+        <v>10.1256</v>
       </c>
     </row>
   </sheetData>
@@ -2026,11 +2308,9 @@
       <c r="D2" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="29"/>
       <c r="M2" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="N2" s="29"/>
       <c r="V2" s="28" t="s">
         <v>25</v>
       </c>
@@ -2101,7 +2381,7 @@
       <c r="V4" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="W4" s="30" t="s">
+      <c r="W4" s="27" t="s">
         <v>22</v>
       </c>
     </row>
@@ -3440,11 +3720,9 @@
       <c r="D2" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="29"/>
       <c r="M2" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="N2" s="29"/>
       <c r="V2" s="28" t="s">
         <v>25</v>
       </c>
@@ -3515,7 +3793,7 @@
       <c r="V4" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="W4" s="30" t="s">
+      <c r="W4" s="27" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>